<commit_message>
Refine New Admiralty buildings from citywalls
- Z136 Большой каменный эллинг: 129 × 35 m, 25 m to the rafters, arched
  ends (citywalls, after M. S. Stiglitz)
- Z160: citywalls and RGIS confirm Главное корабельное здание, a two-storey
  workshop with a clock tower built up to four storeys
- Z161 Караульный дом: rebuilt as a two-storey building
- Y6ea82e: names, dates and status from citywalls
- README: citywalls sources; photos and RGIS plan fragments are on
  p0–p3.citywalls.ru

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012YqYbaVT5dEygR6d1pcCPo
</commit_message>
<xml_diff>
--- a/admiralty-shipyards-territory/dist/admiralty-shipyards-registry.xlsx
+++ b/admiralty-shipyards-territory/dist/admiralty-shipyards-registry.xlsx
@@ -8346,7 +8346,7 @@
         <v>1</v>
       </c>
       <c r="F142">
-        <v>31.5</v>
+        <v>33</v>
       </c>
       <c r="G142" s="3">
         <v>4937</v>
@@ -8355,7 +8355,7 @@
         <v>4937</v>
       </c>
       <c r="I142" s="3">
-        <v>147040</v>
+        <v>154445</v>
       </c>
       <c r="W142" t="inlineStr">
         <is>
@@ -14876,7 +14876,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t xml:space="preserve">Караульный дом</t>
+          <t xml:space="preserve">Караульный дом (северная проходная Нового Адмиралтейства)</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -14890,19 +14890,19 @@
         </is>
       </c>
       <c r="E256">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F256">
-        <v>7</v>
+        <v>11.5</v>
       </c>
       <c r="G256">
         <v>157</v>
       </c>
       <c r="H256">
-        <v>157</v>
-      </c>
-      <c r="I256">
-        <v>785</v>
+        <v>314</v>
+      </c>
+      <c r="I256" s="3">
+        <v>1491</v>
       </c>
       <c r="W256" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix broken flat roofs and flagged yard buildings
- Flat roofs: the parapet inset is checked and falls back to a smaller
  inset or a plain roof, so roofs no longer cross the walls on complex
  outlines (Z55, Z118, Z148, Ybea863, Y40444c and others); self-intersecting
  outlines are cleaned; check.mjs flags roofs outside the outline
- Z27: one-storey checkpoint wing; Z77: three storeys, low first-floor
  windows (`sill`), not taller than Z75; Z76 and Z47 from a photo
  identified on site; Z148, Ybea863, Y40444c get clean outlines
- custom.json parts take `type`; editor field for first-floor sill height
- references: Z76 photo, PastVu views around Berdov bridge

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012YqYbaVT5dEygR6d1pcCPo
</commit_message>
<xml_diff>
--- a/admiralty-shipyards-territory/dist/admiralty-shipyards-registry.xlsx
+++ b/admiralty-shipyards-territory/dist/admiralty-shipyards-registry.xlsx
@@ -799,10 +799,10 @@
         <v>1338</v>
       </c>
       <c r="H11" s="3">
-        <v>6691</v>
+        <v>5200</v>
       </c>
       <c r="I11" s="3">
-        <v>23551</v>
+        <v>18485</v>
       </c>
       <c r="W11" t="inlineStr">
         <is>
@@ -3762,17 +3762,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Z121</t>
+          <t xml:space="preserve">Ybea863</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Административно-бытовой корпус</t>
+          <t xml:space="preserve">Склад</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Административно-бытовой корпус</t>
+          <t xml:space="preserve">Склад</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -3781,19 +3781,19 @@
         </is>
       </c>
       <c r="E63">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F63">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="G63">
-        <v>814</v>
-      </c>
-      <c r="H63" s="3">
-        <v>2443</v>
+        <v>856</v>
+      </c>
+      <c r="H63">
+        <v>856</v>
       </c>
       <c r="I63" s="3">
-        <v>9773</v>
+        <v>7701</v>
       </c>
       <c r="W63" t="inlineStr">
         <is>
@@ -3807,30 +3807,30 @@
       </c>
       <c r="Y63" t="inlineStr">
         <is>
-          <t xml:space="preserve">OpenStreetMap</t>
+          <t xml:space="preserve">Microsoft ML Buildings</t>
         </is>
       </c>
       <c r="Z63">
-        <v>59.922568</v>
+        <v>59.926101</v>
       </c>
       <c r="AA63">
-        <v>30.274415</v>
+        <v>30.275729</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ybea863</t>
+          <t xml:space="preserve">Z121</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Склад</t>
+          <t xml:space="preserve">Административно-бытовой корпус</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Склад</t>
+          <t xml:space="preserve">Административно-бытовой корпус</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -3839,19 +3839,19 @@
         </is>
       </c>
       <c r="E64">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F64">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="G64">
-        <v>809</v>
-      </c>
-      <c r="H64">
-        <v>809</v>
+        <v>814</v>
+      </c>
+      <c r="H64" s="3">
+        <v>2443</v>
       </c>
       <c r="I64" s="3">
-        <v>7284</v>
+        <v>9773</v>
       </c>
       <c r="W64" t="inlineStr">
         <is>
@@ -3865,14 +3865,14 @@
       </c>
       <c r="Y64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Microsoft ML Buildings</t>
+          <t xml:space="preserve">OpenStreetMap</t>
         </is>
       </c>
       <c r="Z64">
-        <v>59.92612</v>
+        <v>59.922568</v>
       </c>
       <c r="AA64">
-        <v>30.275704</v>
+        <v>30.274415</v>
       </c>
     </row>
     <row r="65">
@@ -3958,16 +3958,16 @@
         <v>1</v>
       </c>
       <c r="F66">
-        <v>9</v>
+        <v>11.5</v>
       </c>
       <c r="G66">
-        <v>661</v>
+        <v>689</v>
       </c>
       <c r="H66">
-        <v>661</v>
+        <v>689</v>
       </c>
       <c r="I66" s="3">
-        <v>5947</v>
+        <v>7060</v>
       </c>
       <c r="W66" t="inlineStr">
         <is>
@@ -3985,10 +3985,10 @@
         </is>
       </c>
       <c r="Z66">
-        <v>59.921845</v>
+        <v>59.921843</v>
       </c>
       <c r="AA66">
-        <v>30.275737</v>
+        <v>30.27575</v>
       </c>
     </row>
     <row r="67">
@@ -4120,7 +4120,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Вспомогательное здание</t>
+          <t xml:space="preserve">Административно-бытовой корпус</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -4129,28 +4129,23 @@
         </is>
       </c>
       <c r="E69">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F69">
-        <v>6.5</v>
+        <v>10.5</v>
       </c>
       <c r="G69">
         <v>536</v>
       </c>
       <c r="H69" s="3">
-        <v>1071</v>
+        <v>1607</v>
       </c>
       <c r="I69" s="3">
-        <v>3482</v>
+        <v>5626</v>
       </c>
       <c r="W69" t="inlineStr">
         <is>
           <t xml:space="preserve">Нет данных</t>
-        </is>
-      </c>
-      <c r="X69" t="inlineStr">
-        <is>
-          <t xml:space="preserve">да</t>
         </is>
       </c>
       <c r="Y69" t="inlineStr">
@@ -8111,28 +8106,23 @@
         </is>
       </c>
       <c r="E138">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F138">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="G138" s="3">
         <v>8440</v>
       </c>
       <c r="H138" s="3">
-        <v>8440</v>
+        <v>25319</v>
       </c>
       <c r="I138" s="3">
-        <v>168794</v>
+        <v>109716</v>
       </c>
       <c r="W138" t="inlineStr">
         <is>
           <t xml:space="preserve">Нет данных</t>
-        </is>
-      </c>
-      <c r="X138" t="inlineStr">
-        <is>
-          <t xml:space="preserve">да</t>
         </is>
       </c>
       <c r="Y138" t="inlineStr">
@@ -9560,17 +9550,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t xml:space="preserve">Z143</t>
+          <t xml:space="preserve">Y40444c</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t xml:space="preserve">Нарядный дом</t>
+          <t xml:space="preserve">Вспомогательное здание</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t xml:space="preserve">Историческое здание</t>
+          <t xml:space="preserve">Вспомогательное здание</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -9582,48 +9572,53 @@
         <v>2</v>
       </c>
       <c r="F164">
-        <v>11.5</v>
+        <v>6.5</v>
       </c>
       <c r="G164">
-        <v>320</v>
+        <v>334</v>
       </c>
       <c r="H164">
-        <v>639</v>
+        <v>668</v>
       </c>
       <c r="I164" s="3">
-        <v>3037</v>
+        <v>2171</v>
       </c>
       <c r="W164" t="inlineStr">
         <is>
           <t xml:space="preserve">Нет данных</t>
         </is>
       </c>
+      <c r="X164" t="inlineStr">
+        <is>
+          <t xml:space="preserve">да</t>
+        </is>
+      </c>
       <c r="Y164" t="inlineStr">
         <is>
-          <t xml:space="preserve">OpenStreetMap</t>
+          <t xml:space="preserve">Microsoft ML Buildings</t>
         </is>
       </c>
       <c r="Z164">
-        <v>59.92917</v>
+        <v>59.931376</v>
       </c>
       <c r="AA164">
-        <v>30.27945</v>
+        <v>30.28093</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t xml:space="preserve">Y40444c</t>
+          <t xml:space="preserve">Z143</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t xml:space="preserve">Вспомогательное здание</t>
+          <t xml:space="preserve">Нарядный дом</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t xml:space="preserve">Вспомогательное здание</t>
+          <t xml:space="preserve">Историческое здание</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -9635,37 +9630,32 @@
         <v>2</v>
       </c>
       <c r="F165">
-        <v>6.5</v>
+        <v>11.5</v>
       </c>
       <c r="G165">
-        <v>306</v>
+        <v>320</v>
       </c>
       <c r="H165">
-        <v>612</v>
+        <v>639</v>
       </c>
       <c r="I165" s="3">
-        <v>1988</v>
+        <v>3037</v>
       </c>
       <c r="W165" t="inlineStr">
         <is>
           <t xml:space="preserve">Нет данных</t>
         </is>
       </c>
-      <c r="X165" t="inlineStr">
-        <is>
-          <t xml:space="preserve">да</t>
-        </is>
-      </c>
       <c r="Y165" t="inlineStr">
         <is>
-          <t xml:space="preserve">Microsoft ML Buildings</t>
+          <t xml:space="preserve">OpenStreetMap</t>
         </is>
       </c>
       <c r="Z165">
-        <v>59.931374</v>
+        <v>59.92917</v>
       </c>
       <c r="AA165">
-        <v>30.28092</v>
+        <v>30.27945</v>
       </c>
     </row>
     <row r="166">

</xml_diff>

<commit_message>
Remove the enterprise map image and every mention of it
The source image data/source/enterprise-map.png and the two tools that read
it (tools/trace_map.py, tools/register_map.py) are deleted. User-visible
text no longer cites an enterprise map: page subtitle and sources note,
building descriptions («Контур — по карте предприятия» dropped), registry
source label and Excel sheet, custom.json notes, promo page and PDF. Code
comments and README speak of the source plan (map-trace.js) neutrally.
Geometry is unchanged: the model is built from the same traced data.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012YqYbaVT5dEygR6d1pcCPo
</commit_message>
<xml_diff>
--- a/admiralty-shipyards-territory/dist/admiralty-shipyards-registry.xlsx
+++ b/admiralty-shipyards-territory/dist/admiralty-shipyards-registry.xlsx
@@ -293,7 +293,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y2">
@@ -409,7 +409,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y4">
@@ -525,7 +525,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y6">
@@ -578,7 +578,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y7">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y15">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y19">
@@ -1438,7 +1438,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y22">
@@ -1496,7 +1496,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y23">
@@ -3115,7 +3115,7 @@
       </c>
       <c r="X51" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y51">
@@ -3168,7 +3168,7 @@
       </c>
       <c r="X52" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y52">
@@ -3226,7 +3226,7 @@
       </c>
       <c r="X53" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y53">
@@ -3342,7 +3342,7 @@
       </c>
       <c r="X55" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y55">
@@ -3400,7 +3400,7 @@
       </c>
       <c r="X56" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y56">
@@ -3632,7 +3632,7 @@
       </c>
       <c r="X60" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y60">
@@ -3917,7 +3917,7 @@
       </c>
       <c r="X65" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y65">
@@ -3975,7 +3975,7 @@
       </c>
       <c r="X66" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y66">
@@ -4144,7 +4144,7 @@
       </c>
       <c r="X69" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y69">
@@ -4318,7 +4318,7 @@
       </c>
       <c r="X72" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y72">
@@ -4376,7 +4376,7 @@
       </c>
       <c r="X73" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y73">
@@ -4434,7 +4434,7 @@
       </c>
       <c r="X74" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y74">
@@ -5072,7 +5072,7 @@
       </c>
       <c r="X85" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y85">
@@ -6580,7 +6580,7 @@
       </c>
       <c r="X111" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y111">
@@ -6686,7 +6686,7 @@
       </c>
       <c r="X113" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y113">
@@ -6850,7 +6850,7 @@
       </c>
       <c r="X116" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y116">
@@ -6903,7 +6903,7 @@
       </c>
       <c r="X117" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y117">
@@ -6956,7 +6956,7 @@
       </c>
       <c r="X118" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y118">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="X119" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y119">
@@ -7067,7 +7067,7 @@
       </c>
       <c r="X120" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y120">
@@ -7125,7 +7125,7 @@
       </c>
       <c r="X121" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y121">
@@ -7294,7 +7294,7 @@
       </c>
       <c r="X124" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y124">
@@ -7637,7 +7637,7 @@
       </c>
       <c r="X130" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y130">
@@ -7975,7 +7975,7 @@
       </c>
       <c r="X136" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y136">
@@ -8033,7 +8033,7 @@
       </c>
       <c r="X137" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y137">
@@ -8550,7 +8550,7 @@
       </c>
       <c r="X146" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y146">
@@ -8724,7 +8724,7 @@
       </c>
       <c r="X149" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y149">
@@ -8956,7 +8956,7 @@
       </c>
       <c r="X153" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y153">
@@ -9246,7 +9246,7 @@
       </c>
       <c r="X158" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y158">
@@ -9304,7 +9304,7 @@
       </c>
       <c r="X159" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y159">
@@ -9362,7 +9362,7 @@
       </c>
       <c r="X160" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y160">
@@ -9589,7 +9589,7 @@
       </c>
       <c r="X164" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y164">
@@ -9647,7 +9647,7 @@
       </c>
       <c r="X165" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y165">
@@ -9763,7 +9763,7 @@
       </c>
       <c r="X167" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y167">
@@ -10744,7 +10744,7 @@
       </c>
       <c r="X184" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y184">
@@ -10797,7 +10797,7 @@
       </c>
       <c r="X185" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y185">
@@ -10850,7 +10850,7 @@
       </c>
       <c r="X186" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y186">
@@ -10903,7 +10903,7 @@
       </c>
       <c r="X187" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y187">
@@ -10956,7 +10956,7 @@
       </c>
       <c r="X188" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y188">
@@ -11009,7 +11009,7 @@
       </c>
       <c r="X189" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y189">
@@ -11289,7 +11289,7 @@
       </c>
       <c r="X194" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y194">
@@ -11801,7 +11801,7 @@
       </c>
       <c r="X203" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y203">
@@ -11975,7 +11975,7 @@
       </c>
       <c r="X206" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y206">
@@ -12207,7 +12207,7 @@
       </c>
       <c r="X210" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y210">
@@ -12429,7 +12429,7 @@
       </c>
       <c r="X214" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y214">
@@ -12661,7 +12661,7 @@
       </c>
       <c r="X218" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y218">
@@ -12951,7 +12951,7 @@
       </c>
       <c r="X223" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y223">
@@ -13183,7 +13183,7 @@
       </c>
       <c r="X227" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y227">
@@ -13294,7 +13294,7 @@
       </c>
       <c r="X229" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y229">
@@ -13352,7 +13352,7 @@
       </c>
       <c r="X230" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y230">
@@ -13811,7 +13811,7 @@
       </c>
       <c r="X238" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y238">
@@ -13869,7 +13869,7 @@
       </c>
       <c r="X239" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y239">
@@ -13985,7 +13985,7 @@
       </c>
       <c r="X241" t="inlineStr">
         <is>
-          <t xml:space="preserve">карта предприятия</t>
+          <t xml:space="preserve">уточнённый контур</t>
         </is>
       </c>
       <c r="Y241">
@@ -17316,7 +17316,7 @@
       </c>
       <c r="B7" t="inlineStr" s="7">
         <is>
-          <t xml:space="preserve">OpenStreetMap и Microsoft ML Buildings (через Overture Maps, лицензия ODbL), карта предприятия.</t>
+          <t xml:space="preserve">OpenStreetMap и Microsoft ML Buildings (через Overture Maps, лицензия ODbL); часть контуров уточнена.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Site data modules: no origin notes anywhere
Data modules renamed to site.js, site-apply.js, site-structures.js and
site-marks.js with matching identifiers. Texts, the Excel help sheet,
README, comments and tests no longer describe where contours, numbers or
inventory data come from; the demo notes say the values are conventional.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012YqYbaVT5dEygR6d1pcCPo
</commit_message>
<xml_diff>
--- a/admiralty-shipyards-territory/dist/admiralty-shipyards-registry.xlsx
+++ b/admiralty-shipyards-territory/dist/admiralty-shipyards-registry.xlsx
@@ -31529,7 +31529,7 @@
       </c>
       <c r="B5" t="inlineStr" s="7">
         <is>
-          <t xml:space="preserve">Впишите данные в столбцы: Инвентарный №, Год постройки, Класс ОПО, Рег. № ОПО, № заключения ЭПБ, Дата заключения ЭПБ, Срок безопасной эксплуатации до, Техническое состояние, Дата обследования, Примечание. Столбец «Код в модели» не меняйте — по нему строки сопоставляются с объектами. Даты — в формате ДД.ММ.ГГГГ. Столбец «Инвентарный №» уже заполнен по данным предприятия, при необходимости поправьте. Затем загрузите файл в реестр кнопкой «Загрузить таблицу».</t>
+          <t xml:space="preserve">Впишите данные в столбцы: Инвентарный №, Год постройки, Класс ОПО, Рег. № ОПО, № заключения ЭПБ, Дата заключения ЭПБ, Срок безопасной эксплуатации до, Техническое состояние, Дата обследования, Примечание. Столбец «Код в модели» не меняйте — по нему строки сопоставляются с объектами. Даты — в формате ДД.ММ.ГГГГ. Столбец «Инвентарный №» уже заполнен, при необходимости поправьте. Затем загрузите файл в реестр кнопкой «Загрузить таблицу».</t>
         </is>
       </c>
     </row>
@@ -31542,18 +31542,6 @@
       <c r="B6" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Площадь застройки — по контуру здания (за вычетом дворов). Этажность — по OpenStreetMap, для цехов и складов без данных — 1, для остальных — по высоте. Общая площадь — площадь застройки × этажность. Строительный объём — площадь застройки × высоту до средней отметки кровли. Высоты цехов верфи в открытых данных отсутствуют и оценены — такие строки отмечены в столбце «Высота оценена».</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Данные предприятия</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Контуры зданий и сооружений верфи, номера объектов, инвентарные номера, литеры и назначение — по данным предприятия. У зданий без обмеров высоты оценены по назначению и размерам (отмечены в столбце «Высота оценена»).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Registry: Excel dropdowns and input checks, validated upload
Exported XLSX now carries Excel data validation: dropdown lists for
"Класс ОПО" and "Техническое состояние", date checks for the date
columns and a 1700-2100 range for "Год постройки".

Uploading a table validates the same fields: list values are matched
case-insensitively (Cyrillic I accepted in Roman numerals), impossible
dates such as 31.02 are rejected instead of rolling over, out-of-range
years are skipped. Skipped values are listed in the registry message.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012YqYbaVT5dEygR6d1pcCPo
</commit_message>
<xml_diff>
--- a/admiralty-shipyards-territory/dist/admiralty-shipyards-registry.xlsx
+++ b/admiralty-shipyards-territory/dist/admiralty-shipyards-registry.xlsx
@@ -31463,6 +31463,30 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AB516"/>
+  <dataValidations count="6">
+    <dataValidation type="whole" operator="between" allowBlank="1" showErrorMessage="1" errorTitle="Число" error="Введите целое число от 1700 до 2100" sqref="P2:P516">
+      <formula1>1700</formula1>
+      <formula2>2100</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Значение не из списка" error="Выберите одно из значений: I, II, III, IV, не ОПО" promptTitle="Класс ОПО" prompt="Выберите значение из списка" sqref="Q2:Q516">
+      <formula1>"I,II,III,IV,не ОПО"</formula1>
+    </dataValidation>
+    <dataValidation type="date" operator="between" allowBlank="1" showErrorMessage="1" errorTitle="Дата" error="Введите дату в формате ДД.ММ.ГГГГ" sqref="T2:T516">
+      <formula1>1</formula1>
+      <formula2>73050</formula2>
+    </dataValidation>
+    <dataValidation type="date" operator="between" allowBlank="1" showErrorMessage="1" errorTitle="Дата" error="Введите дату в формате ДД.ММ.ГГГГ" sqref="U2:U516">
+      <formula1>1</formula1>
+      <formula2>73050</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Значение не из списка" error="Выберите одно из значений: нормативное, работоспособное, ограниченно работоспособное, аварийное" promptTitle="Техническое состояние" prompt="Выберите значение из списка" sqref="V2:V516">
+      <formula1>"нормативное,работоспособное,ограниченно работоспособное,аварийное"</formula1>
+    </dataValidation>
+    <dataValidation type="date" operator="between" allowBlank="1" showErrorMessage="1" errorTitle="Дата" error="Введите дату в формате ДД.ММ.ГГГГ" sqref="W2:W516">
+      <formula1>1</formula1>
+      <formula2>73050</formula2>
+    </dataValidation>
+  </dataValidations>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Registry XLSX: yellow headers for fill-in columns, dropdown note in help
Columns the maintenance service fills in get a yellow header so they
are easy to spot; the header row is taller and the date columns wider
so no header is cut off. The help sheet explains where the dropdown
lists are and that values not from the list are skipped on upload.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012YqYbaVT5dEygR6d1pcCPo
</commit_message>
<xml_diff>
--- a/admiralty-shipyards-territory/dist/admiralty-shipyards-registry.xlsx
+++ b/admiralty-shipyards-territory/dist/admiralty-shipyards-registry.xlsx
@@ -27,7 +27,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -54,6 +54,11 @@
         <fgColor rgb="FFCDEBD6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -67,7 +72,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1" vertical="center"/>
@@ -79,6 +84,9 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -109,10 +117,10 @@
     <col min="17" max="17" width="18" customWidth="1"/>
     <col min="18" max="18" width="18" customWidth="1"/>
     <col min="19" max="19" width="18" customWidth="1"/>
-    <col min="20" max="20" width="14" customWidth="1"/>
-    <col min="21" max="21" width="14" customWidth="1"/>
+    <col min="20" max="20" width="18" customWidth="1"/>
+    <col min="21" max="21" width="18" customWidth="1"/>
     <col min="22" max="22" width="18" customWidth="1"/>
-    <col min="23" max="23" width="14" customWidth="1"/>
+    <col min="23" max="23" width="18" customWidth="1"/>
     <col min="24" max="24" width="30" customWidth="1"/>
     <col min="25" max="25" width="14" customWidth="1"/>
     <col min="26" max="26" width="12" customWidth="1"/>
@@ -120,7 +128,7 @@
     <col min="28" max="28" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="45" customHeight="1">
       <c r="A1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Код в модели</t>
@@ -136,7 +144,7 @@
           <t xml:space="preserve">№ объекта</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr" s="1">
+      <c r="D1" t="inlineStr" s="8">
         <is>
           <t xml:space="preserve">Инвентарный №</t>
         </is>
@@ -196,47 +204,47 @@
           <t xml:space="preserve">Отвечает за здание</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr" s="1">
+      <c r="P1" t="inlineStr" s="8">
         <is>
           <t xml:space="preserve">Год постройки</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr" s="1">
+      <c r="Q1" t="inlineStr" s="8">
         <is>
           <t xml:space="preserve">Класс ОПО</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr" s="1">
+      <c r="R1" t="inlineStr" s="8">
         <is>
           <t xml:space="preserve">Рег. № ОПО</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr" s="1">
+      <c r="S1" t="inlineStr" s="8">
         <is>
           <t xml:space="preserve">№ заключения ЭПБ</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr" s="1">
+      <c r="T1" t="inlineStr" s="8">
         <is>
           <t xml:space="preserve">Дата заключения ЭПБ</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr" s="1">
+      <c r="U1" t="inlineStr" s="8">
         <is>
           <t xml:space="preserve">Срок безопасной эксплуатации до</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr" s="1">
+      <c r="V1" t="inlineStr" s="8">
         <is>
           <t xml:space="preserve">Техническое состояние</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr" s="1">
+      <c r="W1" t="inlineStr" s="8">
         <is>
           <t xml:space="preserve">Дата обследования</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr" s="1">
+      <c r="X1" t="inlineStr" s="8">
         <is>
           <t xml:space="preserve">Примечание</t>
         </is>
@@ -31497,7 +31505,7 @@
     <col min="2" max="2" width="110" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="45" customHeight="1">
       <c r="A1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Параметр</t>
@@ -31553,17 +31561,29 @@
       </c>
       <c r="B5" t="inlineStr" s="7">
         <is>
-          <t xml:space="preserve">Впишите данные в столбцы: Инвентарный №, Год постройки, Класс ОПО, Рег. № ОПО, № заключения ЭПБ, Дата заключения ЭПБ, Срок безопасной эксплуатации до, Техническое состояние, Дата обследования, Примечание. Столбец «Код в модели» не меняйте — по нему строки сопоставляются с объектами. Даты — в формате ДД.ММ.ГГГГ. Столбец «Инвентарный №» уже заполнен, при необходимости поправьте. Затем загрузите файл в реестр кнопкой «Загрузить таблицу».</t>
+          <t xml:space="preserve">Впишите данные в столбцы с жёлтой шапкой: Инвентарный №, Год постройки, Класс ОПО, Рег. № ОПО, № заключения ЭПБ, Дата заключения ЭПБ, Срок безопасной эксплуатации до, Техническое состояние, Дата обследования, Примечание. Столбец «Код в модели» не меняйте — по нему строки сопоставляются с объектами. Даты — в формате ДД.ММ.ГГГГ. Столбец «Инвентарный №» уже заполнен, при необходимости поправьте. Затем загрузите файл в реестр кнопкой «Загрузить таблицу».</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t xml:space="preserve">Выпадающие списки</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">В столбцах «Класс ОПО» и «Техническое состояние» значение выбирается из списка: выделите ячейку и нажмите стрелку справа от неё. Если Excel открыл файл в режиме защищённого просмотра, сначала нажмите «Разрешить редактирование». Значения не из списка, неверные даты и год постройки вне 1700–2100 при загрузке в реестр пропускаются.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t xml:space="preserve">Расчётные показатели</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr" s="7">
+      <c r="B7" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Площадь застройки — по контуру здания (за вычетом дворов). Этажность — по OpenStreetMap, для цехов и складов без данных — 1, для остальных — по высоте. Общая площадь — площадь застройки × этажность. Строительный объём — площадь застройки × высоту до средней отметки кровли. Высоты цехов верфи в открытых данных отсутствуют и оценены — такие строки отмечены в столбце «Высота оценена».</t>
         </is>

</xml_diff>

<commit_message>
Perimeter from street views: stucco wall with arches, buildings by photos
Fences along the Pryazhka embankment, Stepan Razin street and Rizhsky
prospekt get a new type: a stucco wall with a plinth, pilasters and a
blind arch in every bay, as the real historic wall looks. The brick
wall stays on the island, concrete panels elsewhere.

Buildings adjusted to street views: building 54 on the Pryazhka
(Z141) is a three-storey yellow block with a hipped roof; admin
building 2 at the south gate (Z65) is dark brick with window bands,
five floors; the guard house at the north gate (G115) is light
stucco; the repair-zone blocks of shop 26 on the island (Z190, Z191),
the boiler house and the old shore buildings get their colours and
floor counts; the corner house at Rizhsky 51 is five floors.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012YqYbaVT5dEygR6d1pcCPo
</commit_message>
<xml_diff>
--- a/admiralty-shipyards-territory/dist/admiralty-shipyards-registry.xlsx
+++ b/admiralty-shipyards-territory/dist/admiralty-shipyards-registry.xlsx
@@ -1058,19 +1058,19 @@
         <v>20.1</v>
       </c>
       <c r="V13">
-        <v>15</v>
+        <v>17.5</v>
       </c>
       <c r="W13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X13" s="3">
         <v>1191</v>
       </c>
       <c r="Y13" s="3">
-        <v>4762</v>
+        <v>5953</v>
       </c>
       <c r="Z13" s="3">
-        <v>17858</v>
+        <v>20835</v>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
@@ -4117,7 +4117,7 @@
         <v>38</v>
       </c>
       <c r="V59">
-        <v>12</v>
+        <v>15.5</v>
       </c>
       <c r="W59">
         <v>3</v>
@@ -4129,7 +4129,7 @@
         <v>3364</v>
       </c>
       <c r="Z59" s="3">
-        <v>13454</v>
+        <v>14762</v>
       </c>
       <c r="AA59" t="inlineStr">
         <is>
@@ -11414,19 +11414,19 @@
         <v>17.3</v>
       </c>
       <c r="V172">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="W172">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="X172" s="3">
         <v>1094</v>
       </c>
       <c r="Y172" s="3">
-        <v>1126</v>
+        <v>3314</v>
       </c>
       <c r="Z172" s="3">
-        <v>7801</v>
+        <v>12178</v>
       </c>
       <c r="AA172" t="inlineStr">
         <is>
@@ -12025,19 +12025,19 @@
         <v>24.7</v>
       </c>
       <c r="V181">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="W181">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X181">
         <v>619</v>
       </c>
       <c r="Y181" s="3">
-        <v>1995</v>
+        <v>2615</v>
       </c>
       <c r="Z181" s="3">
-        <v>8049</v>
+        <v>9288</v>
       </c>
       <c r="AA181" t="inlineStr">
         <is>
@@ -12350,7 +12350,7 @@
         <v>23.5</v>
       </c>
       <c r="V186">
-        <v>7.6</v>
+        <v>8.2</v>
       </c>
       <c r="W186">
         <v>2</v>
@@ -12362,7 +12362,7 @@
         <v>1043</v>
       </c>
       <c r="Z186" s="3">
-        <v>3983</v>
+        <v>4283</v>
       </c>
       <c r="AA186" t="inlineStr">
         <is>
@@ -12885,13 +12885,13 @@
         <v>7</v>
       </c>
       <c r="W194">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X194">
         <v>357</v>
       </c>
       <c r="Y194">
-        <v>357</v>
+        <v>713</v>
       </c>
       <c r="Z194" s="3">
         <v>2497</v>
@@ -13018,13 +13018,13 @@
         <v>9</v>
       </c>
       <c r="W196">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X196">
         <v>334</v>
       </c>
       <c r="Y196">
-        <v>400</v>
+        <v>734</v>
       </c>
       <c r="Z196" s="3">
         <v>3304</v>
@@ -13240,13 +13240,13 @@
         <v>9</v>
       </c>
       <c r="W199">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X199">
         <v>304</v>
       </c>
       <c r="Y199">
-        <v>306</v>
+        <v>610</v>
       </c>
       <c r="Z199" s="3">
         <v>2744</v>
@@ -13296,7 +13296,7 @@
         <v>17.8</v>
       </c>
       <c r="V200">
-        <v>7.6</v>
+        <v>8.2</v>
       </c>
       <c r="W200">
         <v>2</v>
@@ -13308,7 +13308,7 @@
         <v>606</v>
       </c>
       <c r="Z200" s="3">
-        <v>2301</v>
+        <v>2483</v>
       </c>
       <c r="AA200" t="inlineStr">
         <is>
@@ -19169,19 +19169,19 @@
         <v>28.1</v>
       </c>
       <c r="V292">
-        <v>7</v>
+        <v>15.5</v>
       </c>
       <c r="W292">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="X292">
         <v>637</v>
       </c>
-      <c r="Y292">
-        <v>842</v>
+      <c r="Y292" s="3">
+        <v>2117</v>
       </c>
       <c r="Z292" s="3">
-        <v>5383</v>
+        <v>9685</v>
       </c>
       <c r="AA292" t="inlineStr">
         <is>

</xml_diff>